<commit_message>
Mapping: bandaid row to re-label Toast 'Asian Chkn Sal' as full name
The Toast item with GUID b89eaa33-7c46-4b86-a10e-7e8528d6220f has
Name = "Asian Chicken Salad (OLO Pairing Choice)" in toastweb but
Toast Menus API + Toast Analytics still return name = "Asian Chkn Sal"
(POS-name field that wasn't updated, or Toast-side cache lag).

Until Toast's data warehouse catches up to the toastweb rename, route
the abbreviated name through AlohaItemName so the menu performance
report displays it consistently with the other Asian Chicken Salad
variants. The mapping does not modify Toast's data — it only re-labels
the rollup parent in our reports. Safe to leave in place even after
Toast catches up.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Updated Mapping Table.xlsx
+++ b/Updated Mapping Table.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1948"/>
+  <dimension ref="A1:J1949"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -68324,6 +68324,49 @@
         </is>
       </c>
     </row>
+    <row r="1949">
+      <c r="A1949" t="inlineStr">
+        <is>
+          <t>1100000011410021019</t>
+        </is>
+      </c>
+      <c r="B1949" t="n">
+        <v>40070119</v>
+      </c>
+      <c r="C1949" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1949" t="inlineStr">
+        <is>
+          <t>Asian Chkn Sal</t>
+        </is>
+      </c>
+      <c r="E1949" t="inlineStr">
+        <is>
+          <t>Asian Chicken Salad (OLO Pairing Choice)</t>
+        </is>
+      </c>
+      <c r="F1949" t="inlineStr">
+        <is>
+          <t>* Consolidated Salads</t>
+        </is>
+      </c>
+      <c r="G1949" t="inlineStr">
+        <is>
+          <t>b89eaa33-7c46-4b86-a10e-7e8528d6220f</t>
+        </is>
+      </c>
+      <c r="H1949" t="inlineStr">
+        <is>
+          <t>ChickenAsianSalad, Guest Count 0.5, * Consolidated Salads</t>
+        </is>
+      </c>
+      <c r="I1949" t="inlineStr">
+        <is>
+          <t>Guest Count 0.5</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>